<commit_message>
new rar with the latest version
</commit_message>
<xml_diff>
--- a/Hero Stats and Abilities.xlsx
+++ b/Hero Stats and Abilities.xlsx
@@ -1,17 +1,25 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
   <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Python\Projects\Rune_snatching_game\Rune_snatching_game\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <bookViews>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12330"/>
+  </bookViews>
   <sheets>
-    <sheet state="visible" name="Dota 2 Hero Stats and Abilities" sheetId="1" r:id="rId5"/>
+    <sheet name="Dota 2 Hero Stats and Abilities" sheetId="1" r:id="rId1"/>
   </sheets>
-  <definedNames/>
-  <calcPr/>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="56">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="58">
   <si>
     <t>Hero</t>
   </si>
@@ -179,20 +187,27 @@
   </si>
   <si>
     <t>"Wait for it... wait for it... dead!"</t>
+  </si>
+  <si>
+    <t>dd rune multiplier</t>
+  </si>
+  <si>
+    <t>normal rune multiplier</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <fonts count="2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
-      <sz val="10.0"/>
+      <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="10"/>
       <color theme="1"/>
       <name val="Arial"/>
       <scheme val="minor"/>
@@ -203,32 +218,39 @@
       <patternFill patternType="none"/>
     </fill>
     <fill>
-      <patternFill patternType="lightGray"/>
+      <patternFill patternType="gray125"/>
     </fill>
   </fills>
   <borders count="1">
-    <border/>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="2">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0"/>
-    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle xfId="0" name="Normal" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
 </file>
 
 <file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
@@ -236,7 +258,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheets">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Sheets">
   <a:themeElements>
     <a:clrScheme name="Sheets">
       <a:dk1>
@@ -426,21 +448,26 @@
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
+  <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
+  <dimension ref="A1:G18"/>
+  <sheetFormatPr defaultColWidth="12.5703125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
-    <col customWidth="1" min="4" max="4" width="38.38"/>
-    <col customWidth="1" min="5" max="5" width="27.25"/>
+    <col min="4" max="4" width="38.42578125" customWidth="1"/>
+    <col min="5" max="5" width="31.28515625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="19" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="15.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -456,16 +483,22 @@
       <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="2">
+      <c r="F1" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
         <v>5</v>
       </c>
       <c r="B2" s="1">
-        <v>8.0</v>
+        <v>8</v>
       </c>
       <c r="C2" s="1">
-        <v>10.0</v>
+        <v>10</v>
       </c>
       <c r="D2" s="1" t="s">
         <v>6</v>
@@ -473,16 +506,22 @@
       <c r="E2" s="1" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="3">
+      <c r="F2">
+        <v>1</v>
+      </c>
+      <c r="G2" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A3" s="1" t="s">
         <v>8</v>
       </c>
       <c r="B3" s="1">
-        <v>5.0</v>
+        <v>5</v>
       </c>
       <c r="C3" s="1">
-        <v>10.0</v>
+        <v>10</v>
       </c>
       <c r="D3" s="1" t="s">
         <v>9</v>
@@ -490,16 +529,22 @@
       <c r="E3" s="1" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="4">
+      <c r="F3">
+        <v>1</v>
+      </c>
+      <c r="G3" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A4" s="1" t="s">
         <v>11</v>
       </c>
       <c r="B4" s="1">
-        <v>6.0</v>
+        <v>6</v>
       </c>
       <c r="C4" s="1">
-        <v>9.0</v>
+        <v>9</v>
       </c>
       <c r="D4" s="1" t="s">
         <v>12</v>
@@ -507,16 +552,22 @@
       <c r="E4" s="1" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="5">
+      <c r="F4">
+        <v>1</v>
+      </c>
+      <c r="G4" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A5" s="1" t="s">
         <v>14</v>
       </c>
       <c r="B5" s="1">
-        <v>5.0</v>
+        <v>5</v>
       </c>
       <c r="C5" s="1">
-        <v>10.0</v>
+        <v>10</v>
       </c>
       <c r="D5" s="1" t="s">
         <v>15</v>
@@ -524,16 +575,22 @@
       <c r="E5" s="1" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="6">
+      <c r="F5">
+        <v>1</v>
+      </c>
+      <c r="G5" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A6" s="1" t="s">
         <v>17</v>
       </c>
       <c r="B6" s="1">
-        <v>4.0</v>
+        <v>4</v>
       </c>
       <c r="C6" s="1">
-        <v>16.0</v>
+        <v>16</v>
       </c>
       <c r="D6" s="1" t="s">
         <v>18</v>
@@ -541,16 +598,22 @@
       <c r="E6" s="1" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="7">
+      <c r="F6">
+        <v>1</v>
+      </c>
+      <c r="G6" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A7" s="1" t="s">
         <v>20</v>
       </c>
       <c r="B7" s="1">
-        <v>6.0</v>
+        <v>6</v>
       </c>
       <c r="C7" s="1">
-        <v>12.0</v>
+        <v>12</v>
       </c>
       <c r="D7" s="1" t="s">
         <v>21</v>
@@ -558,16 +621,22 @@
       <c r="E7" s="1" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="8">
+      <c r="F7">
+        <v>1</v>
+      </c>
+      <c r="G7" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A8" s="1" t="s">
         <v>23</v>
       </c>
       <c r="B8" s="1">
-        <v>6.0</v>
+        <v>6</v>
       </c>
       <c r="C8" s="1">
-        <v>10.0</v>
+        <v>10</v>
       </c>
       <c r="D8" s="1" t="s">
         <v>24</v>
@@ -575,16 +644,22 @@
       <c r="E8" s="1" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="9">
+      <c r="F8">
+        <v>1</v>
+      </c>
+      <c r="G8" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A9" s="1" t="s">
         <v>26</v>
       </c>
       <c r="B9" s="1">
-        <v>7.0</v>
+        <v>7</v>
       </c>
       <c r="C9" s="1">
-        <v>10.0</v>
+        <v>10</v>
       </c>
       <c r="D9" s="1" t="s">
         <v>27</v>
@@ -592,16 +667,22 @@
       <c r="E9" s="1" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="10">
+      <c r="F9">
+        <v>1</v>
+      </c>
+      <c r="G9" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A10" s="1" t="s">
         <v>29</v>
       </c>
       <c r="B10" s="1">
-        <v>4.0</v>
+        <v>4</v>
       </c>
       <c r="C10" s="1">
-        <v>14.0</v>
+        <v>14</v>
       </c>
       <c r="D10" s="1" t="s">
         <v>30</v>
@@ -609,16 +690,22 @@
       <c r="E10" s="1" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="11">
+      <c r="F10">
+        <v>1</v>
+      </c>
+      <c r="G10" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A11" s="1" t="s">
         <v>32</v>
       </c>
       <c r="B11" s="1">
-        <v>6.0</v>
+        <v>6</v>
       </c>
       <c r="C11" s="1">
-        <v>10.0</v>
+        <v>10</v>
       </c>
       <c r="D11" s="1" t="s">
         <v>33</v>
@@ -626,16 +713,22 @@
       <c r="E11" s="1" t="s">
         <v>34</v>
       </c>
-    </row>
-    <row r="12">
+      <c r="F11">
+        <v>1</v>
+      </c>
+      <c r="G11" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A12" s="1" t="s">
         <v>35</v>
       </c>
       <c r="B12" s="1">
-        <v>8.0</v>
+        <v>8</v>
       </c>
       <c r="C12" s="1">
-        <v>9.0</v>
+        <v>9</v>
       </c>
       <c r="D12" s="1" t="s">
         <v>36</v>
@@ -643,16 +736,22 @@
       <c r="E12" s="1" t="s">
         <v>37</v>
       </c>
-    </row>
-    <row r="13">
+      <c r="F12">
+        <v>1</v>
+      </c>
+      <c r="G12" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A13" s="1" t="s">
         <v>38</v>
       </c>
       <c r="B13" s="1">
-        <v>9.0</v>
+        <v>9</v>
       </c>
       <c r="C13" s="1">
-        <v>10.0</v>
+        <v>10</v>
       </c>
       <c r="D13" s="1" t="s">
         <v>39</v>
@@ -660,16 +759,22 @@
       <c r="E13" s="1" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="14">
+      <c r="F13">
+        <v>1</v>
+      </c>
+      <c r="G13" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A14" s="1" t="s">
         <v>41</v>
       </c>
       <c r="B14" s="1">
-        <v>7.0</v>
+        <v>7</v>
       </c>
       <c r="C14" s="1">
-        <v>8.0</v>
+        <v>8</v>
       </c>
       <c r="D14" s="1" t="s">
         <v>42</v>
@@ -677,16 +782,22 @@
       <c r="E14" s="1" t="s">
         <v>43</v>
       </c>
-    </row>
-    <row r="15">
+      <c r="F14">
+        <v>1</v>
+      </c>
+      <c r="G14" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A15" s="1" t="s">
         <v>44</v>
       </c>
       <c r="B15" s="1">
-        <v>4.0</v>
+        <v>4</v>
       </c>
       <c r="C15" s="1">
-        <v>18.0</v>
+        <v>18</v>
       </c>
       <c r="D15" s="1" t="s">
         <v>45</v>
@@ -694,16 +805,22 @@
       <c r="E15" s="1" t="s">
         <v>46</v>
       </c>
-    </row>
-    <row r="16">
+      <c r="F15">
+        <v>1</v>
+      </c>
+      <c r="G15" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A16" s="1" t="s">
         <v>47</v>
       </c>
       <c r="B16" s="1">
-        <v>5.0</v>
+        <v>5</v>
       </c>
       <c r="C16" s="1">
-        <v>12.0</v>
+        <v>12</v>
       </c>
       <c r="D16" s="1" t="s">
         <v>48</v>
@@ -711,16 +828,22 @@
       <c r="E16" s="1" t="s">
         <v>49</v>
       </c>
-    </row>
-    <row r="17">
+      <c r="F16">
+        <v>1</v>
+      </c>
+      <c r="G16" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A17" s="1" t="s">
         <v>50</v>
       </c>
       <c r="B17" s="1">
-        <v>5.0</v>
+        <v>5</v>
       </c>
       <c r="C17" s="1">
-        <v>11.0</v>
+        <v>11</v>
       </c>
       <c r="D17" s="1" t="s">
         <v>51</v>
@@ -728,16 +851,22 @@
       <c r="E17" s="1" t="s">
         <v>52</v>
       </c>
-    </row>
-    <row r="18">
+      <c r="F17">
+        <v>1</v>
+      </c>
+      <c r="G17" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A18" s="1" t="s">
         <v>53</v>
       </c>
       <c r="B18" s="1">
-        <v>6.0</v>
+        <v>6</v>
       </c>
       <c r="C18" s="1">
-        <v>10.0</v>
+        <v>10</v>
       </c>
       <c r="D18" s="1" t="s">
         <v>54</v>
@@ -745,8 +874,14 @@
       <c r="E18" s="1" t="s">
         <v>55</v>
       </c>
+      <c r="F18">
+        <v>1</v>
+      </c>
+      <c r="G18" s="1">
+        <v>1</v>
+      </c>
     </row>
   </sheetData>
-  <drawing r:id="rId1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
main game hero stats implemented
</commit_message>
<xml_diff>
--- a/Hero Stats and Abilities.xlsx
+++ b/Hero Stats and Abilities.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\a1051243\PyCharmMiscProject\Rune_snatching_game\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7F993B98-1F3D-4AA9-8EE3-E3FFF701A731}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{58BD888D-2936-412D-ADC2-BAE091AB1AF9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Dota 2 Hero Stats and Abilities" sheetId="1" r:id="rId1"/>
@@ -1026,7 +1026,7 @@
         <v>37</v>
       </c>
       <c r="F14">
-        <v>1.5</v>
+        <v>1.1499999999999999</v>
       </c>
       <c r="G14" s="1">
         <v>1</v>

</xml_diff>

<commit_message>
Miss chance and Cave Guardians fight updates
CM Persona and Viper miss chance fix
Added heroes ultimates logic to Cave Guardians fight
</commit_message>
<xml_diff>
--- a/Hero Stats and Abilities.xlsx
+++ b/Hero Stats and Abilities.xlsx
@@ -1,15 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Python\Projects\Rune_snatching_game\Rune_snatching_game\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\a1051243\PyCharmMiscProject\Rune_snatching_game\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D9FB181C-F45D-480A-B3E6-1D300E48824A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-105" yWindow="-105" windowWidth="23250" windowHeight="13890"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Dota 2 Hero Stats and Abilities" sheetId="1" r:id="rId1"/>
@@ -19,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="81" uniqueCount="81">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="81" uniqueCount="79">
   <si>
     <t>Hero</t>
   </si>
@@ -226,9 +227,6 @@
     <t>1 dmg. 15% chance to do 2 dmg</t>
   </si>
   <si>
-    <t>1dmg per sec for 3 sec</t>
-  </si>
-  <si>
     <t>Fatal Bonds: 1.7x Gold from Double Damage runes.</t>
   </si>
   <si>
@@ -238,18 +236,9 @@
     <t>2 dmg per sec to the boss for 3 sec.</t>
   </si>
   <si>
-    <t>boss gets 1 gmd every 5 sec</t>
-  </si>
-  <si>
     <t>heal for 3 hp</t>
   </si>
   <si>
-    <t>.</t>
-  </si>
-  <si>
-    <t>Snipe - huge dmg</t>
-  </si>
-  <si>
     <t>Take Aim: Gold runes are worth +15% gold.</t>
   </si>
   <si>
@@ -259,16 +248,22 @@
     <t>Live drain - gain 1 hp per sec for 4 sec</t>
   </si>
   <si>
-    <t>Corrosive Skin: 18% chance the creep to die (does no dmg)</t>
-  </si>
-  <si>
-    <t>Wolf's Agility: harder to hit creeps. 18% attack against it to miss</t>
+    <t>Wolf's Agility: harder to hit creeps. 20% attack against it to miss</t>
+  </si>
+  <si>
+    <t>Corrosive Skin: 20% chance the creep to die (does no dmg)</t>
+  </si>
+  <si>
+    <t>1dmg per sec for 5 sec</t>
+  </si>
+  <si>
+    <t>boss gets 1 gmd every 4 sec</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
@@ -538,22 +533,22 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
   <dimension ref="A1:K18"/>
-  <sheetFormatPr defaultColWidth="12.5703125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="12.5546875" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="4" max="4" width="53.7109375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="31.28515625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="53.6640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="31.33203125" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="19" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="15.28515625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="14.42578125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="16.140625" customWidth="1"/>
+    <col min="7" max="7" width="15.33203125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="14.44140625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="16.109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" s="6" customFormat="1" ht="38.25" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:11" s="6" customFormat="1" ht="39.6" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
@@ -588,7 +583,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="2" spans="1:11" ht="51" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:11" ht="39.6" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>5</v>
       </c>
@@ -623,7 +618,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="3" spans="1:11" ht="38.25" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:11" ht="39.6" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>8</v>
       </c>
@@ -658,7 +653,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="4" spans="1:11" ht="25.5" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:11" ht="26.4" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>11</v>
       </c>
@@ -669,7 +664,7 @@
         <v>8</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>80</v>
+        <v>75</v>
       </c>
       <c r="E4" s="1" t="s">
         <v>12</v>
@@ -693,7 +688,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="5" spans="1:11" ht="25.5" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:11" ht="26.4" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>13</v>
       </c>
@@ -728,7 +723,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="6" spans="1:11" ht="51" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:11" ht="52.8" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
         <v>16</v>
       </c>
@@ -763,7 +758,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="7" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
         <v>19</v>
       </c>
@@ -798,7 +793,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="8" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
         <v>22</v>
       </c>
@@ -827,13 +822,13 @@
         <v>2</v>
       </c>
       <c r="J8" s="2" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="K8" s="1">
         <v>3</v>
       </c>
     </row>
-    <row r="9" spans="1:11" ht="38.25" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:11" ht="39.6" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
         <v>25</v>
       </c>
@@ -868,7 +863,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="10" spans="1:11" ht="25.5" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:11" ht="26.4" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
         <v>27</v>
       </c>
@@ -894,16 +889,16 @@
         <v>1</v>
       </c>
       <c r="I10" s="1">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J10" s="2" t="s">
-        <v>72</v>
+        <v>78</v>
       </c>
       <c r="K10" s="1">
         <v>4</v>
       </c>
     </row>
-    <row r="11" spans="1:11" ht="63.75" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:11" ht="66" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
         <v>29</v>
       </c>
@@ -929,7 +924,7 @@
         <v>1</v>
       </c>
       <c r="I11" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J11" s="2" t="s">
         <v>64</v>
@@ -938,7 +933,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="12" spans="1:11" ht="25.5" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:11" ht="26.4" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
         <v>31</v>
       </c>
@@ -966,14 +961,14 @@
       <c r="I12" s="1">
         <v>5</v>
       </c>
-      <c r="J12" s="2" t="s">
-        <v>74</v>
+      <c r="J12" t="s">
+        <v>54</v>
       </c>
       <c r="K12" s="1">
         <v>4</v>
       </c>
     </row>
-    <row r="13" spans="1:11" ht="51" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:11" ht="52.8" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
         <v>33</v>
       </c>
@@ -1002,13 +997,13 @@
         <v>3</v>
       </c>
       <c r="J13" s="2" t="s">
-        <v>77</v>
+        <v>73</v>
       </c>
       <c r="K13" s="1">
         <v>3</v>
       </c>
     </row>
-    <row r="14" spans="1:11" ht="38.25" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:11" ht="39.6" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
         <v>36</v>
       </c>
@@ -1019,7 +1014,7 @@
         <v>8</v>
       </c>
       <c r="D14" s="1" t="s">
-        <v>76</v>
+        <v>72</v>
       </c>
       <c r="E14" s="1" t="s">
         <v>37</v>
@@ -1036,14 +1031,14 @@
       <c r="I14" s="1">
         <v>5</v>
       </c>
-      <c r="J14" s="2" t="s">
-        <v>75</v>
+      <c r="J14" t="s">
+        <v>54</v>
       </c>
       <c r="K14" s="1">
         <v>4</v>
       </c>
     </row>
-    <row r="15" spans="1:11" ht="38.25" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:11" ht="39.6" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
         <v>38</v>
       </c>
@@ -1072,13 +1067,13 @@
         <v>1</v>
       </c>
       <c r="J15" s="2" t="s">
-        <v>78</v>
+        <v>74</v>
       </c>
       <c r="K15">
         <v>3</v>
       </c>
     </row>
-    <row r="16" spans="1:11" ht="25.5" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:11" ht="26.4" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
         <v>41</v>
       </c>
@@ -1089,7 +1084,7 @@
         <v>10</v>
       </c>
       <c r="D16" s="1" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="E16" s="1" t="s">
         <v>42</v>
@@ -1107,13 +1102,13 @@
         <v>2</v>
       </c>
       <c r="J16" s="2" t="s">
-        <v>68</v>
+        <v>77</v>
       </c>
       <c r="K16" s="1">
         <v>4</v>
       </c>
     </row>
-    <row r="17" spans="1:11" ht="38.25" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:11" ht="39.6" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
         <v>43</v>
       </c>
@@ -1124,7 +1119,7 @@
         <v>10</v>
       </c>
       <c r="D17" s="1" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="E17" s="1" t="s">
         <v>44</v>
@@ -1142,13 +1137,13 @@
         <v>2</v>
       </c>
       <c r="J17" s="2" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="K17" s="1">
         <v>4</v>
       </c>
     </row>
-    <row r="18" spans="1:11" ht="38.25" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:11" ht="39.6" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
         <v>45</v>
       </c>
@@ -1174,10 +1169,10 @@
         <v>1</v>
       </c>
       <c r="I18" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J18" s="3" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="K18" s="1">
         <v>4</v>

</xml_diff>